<commit_message>
Compounding 2% risk - 206% return 6 months confirmed
</commit_message>
<xml_diff>
--- a/data/backtest_1mo.xlsx
+++ b/data/backtest_1mo.xlsx
@@ -501,10 +501,10 @@
         <v>4673.294</v>
       </c>
       <c r="G2" t="n">
-        <v>4677.426000000001</v>
+        <v>4676.393000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -512,10 +512,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>-20.66</v>
+        <v>-103.3</v>
       </c>
       <c r="K2" t="n">
-        <v>9979.34</v>
+        <v>9896.700000000001</v>
       </c>
     </row>
     <row r="3">
@@ -542,10 +542,10 @@
         <v>4739.909</v>
       </c>
       <c r="G3" t="n">
-        <v>4735.909</v>
+        <v>4736.909</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -553,10 +553,10 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K3" t="n">
-        <v>9959.34</v>
+        <v>9796.700000000001</v>
       </c>
     </row>
     <row r="4">
@@ -583,10 +583,10 @@
         <v>4684.938</v>
       </c>
       <c r="G4" t="n">
-        <v>4688.938</v>
+        <v>4687.938</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -594,10 +594,10 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K4" t="n">
-        <v>9939.34</v>
+        <v>9696.700000000001</v>
       </c>
     </row>
     <row r="5">
@@ -624,21 +624,21 @@
         <v>4704.15</v>
       </c>
       <c r="G5" t="n">
-        <v>4697.186</v>
+        <v>4698.927</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>-34.82</v>
+        <v>348.2</v>
       </c>
       <c r="K5" t="n">
-        <v>9904.52</v>
+        <v>10044.9</v>
       </c>
     </row>
     <row r="6">
@@ -665,10 +665,10 @@
         <v>4683.757</v>
       </c>
       <c r="G6" t="n">
-        <v>4687.757</v>
+        <v>4686.757</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="K6" t="n">
-        <v>9964.52</v>
+        <v>10244.9</v>
       </c>
     </row>
     <row r="7">
@@ -706,10 +706,10 @@
         <v>4692.823</v>
       </c>
       <c r="G7" t="n">
-        <v>4686.058999999997</v>
+        <v>4687.749999999998</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>-33.82</v>
+        <v>-169.1</v>
       </c>
       <c r="K7" t="n">
-        <v>9930.700000000001</v>
+        <v>10075.8</v>
       </c>
     </row>
     <row r="8">
@@ -747,10 +747,10 @@
         <v>4692.28</v>
       </c>
       <c r="G8" t="n">
-        <v>4688.28</v>
+        <v>4689.28</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -758,10 +758,10 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="K8" t="n">
-        <v>9990.700000000001</v>
+        <v>10275.8</v>
       </c>
     </row>
     <row r="9">
@@ -788,10 +788,10 @@
         <v>4554.162</v>
       </c>
       <c r="G9" t="n">
-        <v>4558.162</v>
+        <v>4557.162</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -799,10 +799,10 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K9" t="n">
-        <v>9970.700000000001</v>
+        <v>10175.8</v>
       </c>
     </row>
     <row r="10">
@@ -829,10 +829,10 @@
         <v>4556.443</v>
       </c>
       <c r="G10" t="n">
-        <v>4560.443</v>
+        <v>4559.443</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -840,10 +840,10 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="K10" t="n">
-        <v>10030.7</v>
+        <v>10375.8</v>
       </c>
     </row>
     <row r="11">
@@ -870,10 +870,10 @@
         <v>4551.477</v>
       </c>
       <c r="G11" t="n">
-        <v>4542.001000000001</v>
+        <v>4544.370000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2</v>
+        <v>0.88</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -881,10 +881,10 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>142.14</v>
+        <v>416.94</v>
       </c>
       <c r="K11" t="n">
-        <v>10172.84</v>
+        <v>10792.74</v>
       </c>
     </row>
     <row r="12">
@@ -911,10 +911,10 @@
         <v>4551.477</v>
       </c>
       <c r="G12" t="n">
-        <v>4545.756999999999</v>
+        <v>4547.186999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -922,10 +922,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>85.8</v>
+        <v>286</v>
       </c>
       <c r="K12" t="n">
-        <v>10258.64</v>
+        <v>11078.74</v>
       </c>
     </row>
     <row r="13">
@@ -952,10 +952,10 @@
         <v>4536.941</v>
       </c>
       <c r="G13" t="n">
-        <v>4546.629000000002</v>
+        <v>4544.207000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2</v>
+        <v>0.91</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -963,10 +963,10 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>-48.44</v>
+        <v>-220.4</v>
       </c>
       <c r="K13" t="n">
-        <v>10210.2</v>
+        <v>10858.34</v>
       </c>
     </row>
     <row r="14">
@@ -993,10 +993,10 @@
         <v>4559.429</v>
       </c>
       <c r="G14" t="n">
-        <v>4555.429</v>
+        <v>4556.429</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1004,10 +1004,10 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K14" t="n">
-        <v>10190.2</v>
+        <v>10758.34</v>
       </c>
     </row>
     <row r="15">
@@ -1034,10 +1034,10 @@
         <v>4541.255</v>
       </c>
       <c r="G15" t="n">
-        <v>4545.255</v>
+        <v>4544.255</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1045,10 +1045,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="K15" t="n">
-        <v>10250.2</v>
+        <v>10958.34</v>
       </c>
     </row>
     <row r="16">
@@ -1075,21 +1075,21 @@
         <v>4542.043</v>
       </c>
       <c r="G16" t="n">
-        <v>4547.099</v>
+        <v>4545.835</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>-25.28</v>
+        <v>252.8</v>
       </c>
       <c r="K16" t="n">
-        <v>10224.92</v>
+        <v>11211.14</v>
       </c>
     </row>
     <row r="17">
@@ -1116,10 +1116,10 @@
         <v>4498.683</v>
       </c>
       <c r="G17" t="n">
-        <v>4488.047000000001</v>
+        <v>4490.706000000001</v>
       </c>
       <c r="H17" t="n">
-        <v>0.2</v>
+        <v>0.84</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1127,10 +1127,10 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>-53.18</v>
+        <v>-223.36</v>
       </c>
       <c r="K17" t="n">
-        <v>10171.74</v>
+        <v>10987.79</v>
       </c>
     </row>
     <row r="18">
@@ -1157,10 +1157,10 @@
         <v>4539.78</v>
       </c>
       <c r="G18" t="n">
-        <v>4529.076000000002</v>
+        <v>4531.752000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2</v>
+        <v>0.82</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>-53.52</v>
+        <v>-219.43</v>
       </c>
       <c r="K18" t="n">
-        <v>10118.22</v>
+        <v>10768.35</v>
       </c>
     </row>
     <row r="19">
@@ -1179,7 +1179,7 @@
         <v>46162.92708333334</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>46162.96875</v>
+        <v>46162.94791666666</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
         <v>4536.78</v>
       </c>
       <c r="G19" t="n">
-        <v>4546.223999999999</v>
+        <v>4543.862999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>0.2</v>
+        <v>0.91</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>-47.22</v>
+        <v>429.7</v>
       </c>
       <c r="K19" t="n">
-        <v>10071</v>
+        <v>11198.06</v>
       </c>
     </row>
     <row r="20">
@@ -1239,10 +1239,10 @@
         <v>4515.922</v>
       </c>
       <c r="G20" t="n">
-        <v>4519.922</v>
+        <v>4518.922</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1250,10 +1250,10 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K20" t="n">
-        <v>10051</v>
+        <v>11098.06</v>
       </c>
     </row>
     <row r="21">
@@ -1280,10 +1280,10 @@
         <v>4506.284</v>
       </c>
       <c r="G21" t="n">
-        <v>4510.284</v>
+        <v>4509.284</v>
       </c>
       <c r="H21" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1291,10 +1291,10 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="K21" t="n">
-        <v>10111</v>
+        <v>11298.06</v>
       </c>
     </row>
     <row r="22">
@@ -1321,10 +1321,10 @@
         <v>4533.314</v>
       </c>
       <c r="G22" t="n">
-        <v>4544.35</v>
+        <v>4541.591</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2</v>
+        <v>0.82</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1332,10 +1332,10 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>-55.18</v>
+        <v>-226.24</v>
       </c>
       <c r="K22" t="n">
-        <v>10055.82</v>
+        <v>11071.82</v>
       </c>
     </row>
     <row r="23">
@@ -1362,10 +1362,10 @@
         <v>4519.633</v>
       </c>
       <c r="G23" t="n">
-        <v>4531.968999999999</v>
+        <v>4528.884999999999</v>
       </c>
       <c r="H23" t="n">
-        <v>0.2</v>
+        <v>0.72</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1373,10 +1373,10 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>-61.68</v>
+        <v>-222.05</v>
       </c>
       <c r="K23" t="n">
-        <v>9994.139999999999</v>
+        <v>10849.77</v>
       </c>
     </row>
     <row r="24">
@@ -1403,10 +1403,10 @@
         <v>4519.324</v>
       </c>
       <c r="G24" t="n">
-        <v>4528.2</v>
+        <v>4525.981</v>
       </c>
       <c r="H24" t="n">
-        <v>0.2</v>
+        <v>0.98</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1414,10 +1414,10 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>133.14</v>
+        <v>434.92</v>
       </c>
       <c r="K24" t="n">
-        <v>10127.28</v>
+        <v>11284.69</v>
       </c>
     </row>
     <row r="25">
@@ -1444,10 +1444,10 @@
         <v>4514.193</v>
       </c>
       <c r="G25" t="n">
-        <v>4518.193</v>
+        <v>4517.193</v>
       </c>
       <c r="H25" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K25" t="n">
-        <v>10107.28</v>
+        <v>11184.69</v>
       </c>
     </row>
     <row r="26">
@@ -1485,10 +1485,10 @@
         <v>4508.619</v>
       </c>
       <c r="G26" t="n">
-        <v>4514.043000000002</v>
+        <v>4512.687000000002</v>
       </c>
       <c r="H26" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1496,10 +1496,10 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>-27.12</v>
+        <v>-135.6</v>
       </c>
       <c r="K26" t="n">
-        <v>10080.16</v>
+        <v>11049.09</v>
       </c>
     </row>
     <row r="27">
@@ -1526,10 +1526,10 @@
         <v>4575.134</v>
       </c>
       <c r="G27" t="n">
-        <v>4571.134</v>
+        <v>4572.134</v>
       </c>
       <c r="H27" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1537,10 +1537,10 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="K27" t="n">
-        <v>10140.16</v>
+        <v>11249.09</v>
       </c>
     </row>
     <row r="28">
@@ -1567,10 +1567,10 @@
         <v>4575.128</v>
       </c>
       <c r="G28" t="n">
-        <v>4566.260000000001</v>
+        <v>4568.477000000001</v>
       </c>
       <c r="H28" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1578,10 +1578,10 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>-44.34</v>
+        <v>-221.7</v>
       </c>
       <c r="K28" t="n">
-        <v>10095.82</v>
+        <v>11027.39</v>
       </c>
     </row>
     <row r="29">
@@ -1608,10 +1608,10 @@
         <v>4542.547</v>
       </c>
       <c r="G29" t="n">
-        <v>4538.547</v>
+        <v>4539.547</v>
       </c>
       <c r="H29" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1619,10 +1619,10 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K29" t="n">
-        <v>10075.82</v>
+        <v>10927.39</v>
       </c>
     </row>
     <row r="30">
@@ -1649,10 +1649,10 @@
         <v>4536.459</v>
       </c>
       <c r="G30" t="n">
-        <v>4528.879000000002</v>
+        <v>4530.774000000001</v>
       </c>
       <c r="H30" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1660,10 +1660,10 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>113.7</v>
+        <v>379</v>
       </c>
       <c r="K30" t="n">
-        <v>10189.52</v>
+        <v>11306.39</v>
       </c>
     </row>
     <row r="31">
@@ -1690,21 +1690,21 @@
         <v>4506.214</v>
       </c>
       <c r="G31" t="n">
-        <v>4512.338</v>
+        <v>4510.807</v>
       </c>
       <c r="H31" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>-30.62</v>
+        <v>306.2</v>
       </c>
       <c r="K31" t="n">
-        <v>10158.9</v>
+        <v>11612.59</v>
       </c>
     </row>
     <row r="32">
@@ -1731,10 +1731,10 @@
         <v>4512.215</v>
       </c>
       <c r="G32" t="n">
-        <v>4504.695</v>
+        <v>4506.575</v>
       </c>
       <c r="H32" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1742,10 +1742,10 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>-37.6</v>
+        <v>-188</v>
       </c>
       <c r="K32" t="n">
-        <v>10121.3</v>
+        <v>11424.59</v>
       </c>
     </row>
     <row r="33">
@@ -1772,10 +1772,10 @@
         <v>4456.992</v>
       </c>
       <c r="G33" t="n">
-        <v>4449.395999999999</v>
+        <v>4451.294999999999</v>
       </c>
       <c r="H33" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1783,10 +1783,10 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>-37.98</v>
+        <v>-189.9</v>
       </c>
       <c r="K33" t="n">
-        <v>10083.32</v>
+        <v>11234.69</v>
       </c>
     </row>
     <row r="34">
@@ -1813,10 +1813,10 @@
         <v>4503.198</v>
       </c>
       <c r="G34" t="n">
-        <v>4499.198</v>
+        <v>4500.198</v>
       </c>
       <c r="H34" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>-20</v>
+        <v>-100</v>
       </c>
       <c r="K34" t="n">
-        <v>10063.32</v>
+        <v>11134.69</v>
       </c>
     </row>
     <row r="35">
@@ -1854,10 +1854,10 @@
         <v>4518.088</v>
       </c>
       <c r="G35" t="n">
-        <v>4511.436000000002</v>
+        <v>4513.099000000001</v>
       </c>
       <c r="H35" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1865,10 +1865,10 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>99.78</v>
+        <v>332.6</v>
       </c>
       <c r="K35" t="n">
-        <v>10163.1</v>
+        <v>11467.29</v>
       </c>
     </row>
     <row r="36">
@@ -1895,10 +1895,10 @@
         <v>4519.299</v>
       </c>
       <c r="G36" t="n">
-        <v>4533.474999999999</v>
+        <v>4529.931</v>
       </c>
       <c r="H36" t="n">
-        <v>0.2</v>
+        <v>0.65</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1906,10 +1906,10 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>-70.88</v>
+        <v>-230.36</v>
       </c>
       <c r="K36" t="n">
-        <v>10092.22</v>
+        <v>11236.93</v>
       </c>
     </row>
     <row r="37">
@@ -1936,10 +1936,10 @@
         <v>4556.219</v>
       </c>
       <c r="G37" t="n">
-        <v>4564.771</v>
+        <v>4562.633</v>
       </c>
       <c r="H37" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -1947,10 +1947,10 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>-42.76</v>
+        <v>-213.8</v>
       </c>
       <c r="K37" t="n">
-        <v>10049.46</v>
+        <v>11023.13</v>
       </c>
     </row>
     <row r="38">
@@ -1977,10 +1977,10 @@
         <v>4516.854</v>
       </c>
       <c r="G38" t="n">
-        <v>4528.014</v>
+        <v>4525.224</v>
       </c>
       <c r="H38" t="n">
-        <v>0.2</v>
+        <v>0.79</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1988,10 +1988,10 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>-55.8</v>
+        <v>-220.41</v>
       </c>
       <c r="K38" t="n">
-        <v>9993.66</v>
+        <v>10802.72</v>
       </c>
     </row>
     <row r="39">
@@ -2018,10 +2018,10 @@
         <v>4498.514</v>
       </c>
       <c r="G39" t="n">
-        <v>4509.750000000001</v>
+        <v>4506.941000000001</v>
       </c>
       <c r="H39" t="n">
-        <v>0.2</v>
+        <v>0.77</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2029,10 +2029,10 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>-56.18</v>
+        <v>-216.29</v>
       </c>
       <c r="K39" t="n">
-        <v>9937.48</v>
+        <v>10586.43</v>
       </c>
     </row>
     <row r="40">
@@ -2059,21 +2059,21 @@
         <v>4489.012</v>
       </c>
       <c r="G40" t="n">
-        <v>4485.012</v>
+        <v>4486.012</v>
       </c>
       <c r="H40" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J40" t="n">
-        <v>-20</v>
+        <v>200</v>
       </c>
       <c r="K40" t="n">
-        <v>9917.48</v>
+        <v>10786.43</v>
       </c>
     </row>
     <row r="41">
@@ -2100,10 +2100,10 @@
         <v>4529.791</v>
       </c>
       <c r="G41" t="n">
-        <v>4517.962999999999</v>
+        <v>4520.919999999999</v>
       </c>
       <c r="H41" t="n">
-        <v>0.2</v>
+        <v>0.73</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2111,10 +2111,10 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>-59.14</v>
+        <v>-215.86</v>
       </c>
       <c r="K41" t="n">
-        <v>9858.34</v>
+        <v>10570.57</v>
       </c>
     </row>
     <row r="42">
@@ -2141,21 +2141,21 @@
         <v>4488.498</v>
       </c>
       <c r="G42" t="n">
-        <v>4494.178</v>
+        <v>4492.758</v>
       </c>
       <c r="H42" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN</t>
         </is>
       </c>
       <c r="J42" t="n">
-        <v>-28.4</v>
+        <v>284</v>
       </c>
       <c r="K42" t="n">
-        <v>9829.940000000001</v>
+        <v>10854.57</v>
       </c>
     </row>
     <row r="43">
@@ -2182,10 +2182,10 @@
         <v>4491.498</v>
       </c>
       <c r="G43" t="n">
-        <v>4475.030000000002</v>
+        <v>4479.147000000002</v>
       </c>
       <c r="H43" t="n">
-        <v>0.2</v>
+        <v>0.53</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2193,10 +2193,10 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>-82.34</v>
+        <v>-218.2</v>
       </c>
       <c r="K43" t="n">
-        <v>9747.6</v>
+        <v>10636.37</v>
       </c>
     </row>
     <row r="44">
@@ -2223,10 +2223,10 @@
         <v>4480.146</v>
       </c>
       <c r="G44" t="n">
-        <v>4462.31</v>
+        <v>4466.769</v>
       </c>
       <c r="H44" t="n">
-        <v>0.2</v>
+        <v>0.48</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2234,10 +2234,10 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>-89.18000000000001</v>
+        <v>-214.03</v>
       </c>
       <c r="K44" t="n">
-        <v>9658.42</v>
+        <v>10422.34</v>
       </c>
     </row>
     <row r="45">
@@ -2264,10 +2264,10 @@
         <v>4477.146</v>
       </c>
       <c r="G45" t="n">
-        <v>4482.898</v>
+        <v>4481.46</v>
       </c>
       <c r="H45" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2275,10 +2275,10 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>86.28</v>
+        <v>287.6</v>
       </c>
       <c r="K45" t="n">
-        <v>9744.700000000001</v>
+        <v>10709.94</v>
       </c>
     </row>
     <row r="46">
@@ -2305,10 +2305,10 @@
         <v>4480.574</v>
       </c>
       <c r="G46" t="n">
-        <v>4486.634000000001</v>
+        <v>4485.119000000001</v>
       </c>
       <c r="H46" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2316,10 +2316,10 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>90.90000000000001</v>
+        <v>303</v>
       </c>
       <c r="K46" t="n">
-        <v>9835.6</v>
+        <v>11012.94</v>
       </c>
     </row>
     <row r="47">
@@ -2346,10 +2346,10 @@
         <v>4460.778</v>
       </c>
       <c r="G47" t="n">
-        <v>4468.985999999999</v>
+        <v>4466.933999999999</v>
       </c>
       <c r="H47" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -2357,10 +2357,10 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>123.12</v>
+        <v>410.4</v>
       </c>
       <c r="K47" t="n">
-        <v>9958.719999999999</v>
+        <v>11423.34</v>
       </c>
     </row>
     <row r="48">
@@ -2387,10 +2387,10 @@
         <v>4454.977</v>
       </c>
       <c r="G48" t="n">
-        <v>4464.077000000002</v>
+        <v>4461.802000000001</v>
       </c>
       <c r="H48" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2398,10 +2398,10 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>-45.5</v>
+        <v>-227.5</v>
       </c>
       <c r="K48" t="n">
-        <v>9913.219999999999</v>
+        <v>11195.84</v>
       </c>
     </row>
     <row r="49">
@@ -2428,10 +2428,10 @@
         <v>4460.778</v>
       </c>
       <c r="G49" t="n">
-        <v>4468.902</v>
+        <v>4466.871</v>
       </c>
       <c r="H49" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2439,10 +2439,10 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>-40.62</v>
+        <v>-203.1</v>
       </c>
       <c r="K49" t="n">
-        <v>9872.6</v>
+        <v>10992.74</v>
       </c>
     </row>
     <row r="50">
@@ -2469,10 +2469,10 @@
         <v>4454.977</v>
       </c>
       <c r="G50" t="n">
-        <v>4464.101</v>
+        <v>4461.82</v>
       </c>
       <c r="H50" t="n">
-        <v>0.2</v>
+        <v>0.96</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -2480,10 +2480,10 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>-45.62</v>
+        <v>-218.98</v>
       </c>
       <c r="K50" t="n">
-        <v>9826.98</v>
+        <v>10773.76</v>
       </c>
     </row>
     <row r="51">
@@ -2510,10 +2510,10 @@
         <v>4432.129</v>
       </c>
       <c r="G51" t="n">
-        <v>4438.836999999999</v>
+        <v>4437.159999999999</v>
       </c>
       <c r="H51" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>100.62</v>
+        <v>335.4</v>
       </c>
       <c r="K51" t="n">
-        <v>9927.6</v>
+        <v>11109.16</v>
       </c>
     </row>
     <row r="52">
@@ -2551,10 +2551,10 @@
         <v>4478.535</v>
       </c>
       <c r="G52" t="n">
-        <v>4471.942999999999</v>
+        <v>4473.590999999999</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -2562,10 +2562,10 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>-32.96</v>
+        <v>-164.8</v>
       </c>
       <c r="K52" t="n">
-        <v>9894.639999999999</v>
+        <v>10944.36</v>
       </c>
     </row>
     <row r="53">
@@ -2592,10 +2592,10 @@
         <v>4455.657</v>
       </c>
       <c r="G53" t="n">
-        <v>4462.625000000001</v>
+        <v>4460.883000000001</v>
       </c>
       <c r="H53" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -2603,10 +2603,10 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>104.52</v>
+        <v>348.4</v>
       </c>
       <c r="K53" t="n">
-        <v>9999.16</v>
+        <v>11292.76</v>
       </c>
     </row>
     <row r="54">
@@ -2633,10 +2633,10 @@
         <v>4446.205</v>
       </c>
       <c r="G54" t="n">
-        <v>4440.288999999999</v>
+        <v>4441.767999999999</v>
       </c>
       <c r="H54" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -2644,10 +2644,10 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>88.73999999999999</v>
+        <v>295.8</v>
       </c>
       <c r="K54" t="n">
-        <v>10087.9</v>
+        <v>11588.56</v>
       </c>
     </row>
     <row r="55">
@@ -2674,10 +2674,10 @@
         <v>4342.699</v>
       </c>
       <c r="G55" t="n">
-        <v>4349.291</v>
+        <v>4347.643</v>
       </c>
       <c r="H55" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -2685,10 +2685,10 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>-32.96</v>
+        <v>-164.8</v>
       </c>
       <c r="K55" t="n">
-        <v>10054.94</v>
+        <v>11423.76</v>
       </c>
     </row>
     <row r="56">
@@ -2715,10 +2715,10 @@
         <v>4321.588</v>
       </c>
       <c r="G56" t="n">
-        <v>4329.932000000001</v>
+        <v>4327.846</v>
       </c>
       <c r="H56" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -2726,10 +2726,10 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>-41.72</v>
+        <v>-208.6</v>
       </c>
       <c r="K56" t="n">
-        <v>10013.22</v>
+        <v>11215.16</v>
       </c>
     </row>
     <row r="57">
@@ -2756,10 +2756,10 @@
         <v>4298.402</v>
       </c>
       <c r="G57" t="n">
-        <v>4304.210000000001</v>
+        <v>4302.758000000001</v>
       </c>
       <c r="H57" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -2767,10 +2767,10 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>87.12</v>
+        <v>290.4</v>
       </c>
       <c r="K57" t="n">
-        <v>10100.34</v>
+        <v>11505.56</v>
       </c>
     </row>
     <row r="58">
@@ -2797,10 +2797,10 @@
         <v>4291.515</v>
       </c>
       <c r="G58" t="n">
-        <v>4300.371</v>
+        <v>4298.157</v>
       </c>
       <c r="H58" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -2808,10 +2808,10 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>132.84</v>
+        <v>442.8</v>
       </c>
       <c r="K58" t="n">
-        <v>10233.18</v>
+        <v>11948.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>